<commit_message>
ultima versio nivell 1 i 2 sprint 10
</commit_message>
<xml_diff>
--- a/Sprint 10/dades_GrupA.xlsx
+++ b/Sprint 10/dades_GrupA.xlsx
@@ -591,7 +591,7 @@
         <v>28055</v>
       </c>
       <c r="P2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -5637,7 +5637,7 @@
         <v>19289</v>
       </c>
       <c r="P67" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
@@ -8515,7 +8515,7 @@
         <v>23672</v>
       </c>
       <c r="P104" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -9217,7 +9217,7 @@
         <v>21116</v>
       </c>
       <c r="P113" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -22277,7 +22277,7 @@
         <v>22942</v>
       </c>
       <c r="P281" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
@@ -32389,7 +32389,7 @@
         <v>25864</v>
       </c>
       <c r="P411" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q411" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Pujar Sprint 11 i algunes modificacions del Sprint10
</commit_message>
<xml_diff>
--- a/Sprint 10/dades_GrupA.xlsx
+++ b/Sprint 10/dades_GrupA.xlsx
@@ -2451,7 +2451,7 @@
         <v>38285</v>
       </c>
       <c r="P26" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -6495,7 +6495,7 @@
         <v>32077</v>
       </c>
       <c r="P78" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
@@ -6885,7 +6885,7 @@
         <v>19292</v>
       </c>
       <c r="P83" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -7197,7 +7197,7 @@
         <v>28425</v>
       </c>
       <c r="P87" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
@@ -7895,7 +7895,7 @@
         <v>26970</v>
       </c>
       <c r="P96" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
@@ -8749,7 +8749,7 @@
         <v>35006</v>
       </c>
       <c r="P107" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
@@ -8983,7 +8983,7 @@
         <v>22216</v>
       </c>
       <c r="P110" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
@@ -15987,7 +15987,7 @@
         <v>27326</v>
       </c>
       <c r="P200" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Q200" t="inlineStr">
         <is>
@@ -16299,7 +16299,7 @@
         <v>30982</v>
       </c>
       <c r="P204" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q204" t="inlineStr">
         <is>
@@ -17769,7 +17769,7 @@
         <v>24770</v>
       </c>
       <c r="P223" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q223" t="inlineStr">
         <is>
@@ -19095,7 +19095,7 @@
         <v>26965</v>
       </c>
       <c r="P240" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q240" t="inlineStr">
         <is>
@@ -21189,7 +21189,7 @@
         <v>33544</v>
       </c>
       <c r="P267" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q267" t="inlineStr">
         <is>
@@ -23209,7 +23209,7 @@
         <v>33181</v>
       </c>
       <c r="P293" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q293" t="inlineStr">
         <is>
@@ -27479,7 +27479,7 @@
         <v>20021</v>
       </c>
       <c r="P348" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q348" t="inlineStr">
         <is>
@@ -28723,7 +28723,7 @@
         <v>37197</v>
       </c>
       <c r="P364" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q364" t="inlineStr">
         <is>
@@ -29191,7 +29191,7 @@
         <v>29522</v>
       </c>
       <c r="P370" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q370" t="inlineStr">
         <is>
@@ -30439,7 +30439,7 @@
         <v>28068</v>
       </c>
       <c r="P386" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q386" t="inlineStr">
         <is>
@@ -32857,7 +32857,7 @@
         <v>37563</v>
       </c>
       <c r="P417" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q417" t="inlineStr">
         <is>
@@ -35423,7 +35423,7 @@
         <v>30613</v>
       </c>
       <c r="P450" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q450" t="inlineStr">
         <is>

</xml_diff>